<commit_message>
Update Broadway Court summary PDF and pro forma XLSX
</commit_message>
<xml_diff>
--- a/pa-partners-new/public/deals/broadway-court-pro-forma.xlsx
+++ b/pa-partners-new/public/deals/broadway-court-pro-forma.xlsx
@@ -429,7 +429,7 @@
         <v>Date:</v>
       </c>
       <c r="B3" t="str">
-        <v>9/26/2025</v>
+        <v>9/28/2025</v>
       </c>
     </row>
     <row r="5">
@@ -559,7 +559,7 @@
         <v>Average Monthly Rent (Per Unit):</v>
       </c>
       <c r="B4">
-        <v>890</v>
+        <v>860</v>
       </c>
     </row>
     <row r="5">
@@ -583,7 +583,7 @@
         <v>Annual Rent Growth:</v>
       </c>
       <c r="B7" s="2">
-        <v>0.045</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="8">
@@ -981,7 +981,7 @@
         <v>Total Project Cost</v>
       </c>
       <c r="B6" s="1">
-        <v>2118500</v>
+        <v>2063500</v>
       </c>
     </row>
     <row r="7">
@@ -989,7 +989,7 @@
         <v>Loan Amount</v>
       </c>
       <c r="B7" s="1">
-        <v>1482950</v>
+        <v>1547625</v>
       </c>
     </row>
     <row r="8">
@@ -997,7 +997,7 @@
         <v>Interest Rate</v>
       </c>
       <c r="B8" s="2">
-        <v>0.068</v>
+        <v>0.0675</v>
       </c>
     </row>
     <row r="9">
@@ -1021,7 +1021,7 @@
         <v>LTV</v>
       </c>
       <c r="B11" s="2">
-        <v>0.7</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="12">
@@ -1061,7 +1061,7 @@
         <v>Year 1 NOI</v>
       </c>
       <c r="B16" s="1">
-        <v>165205</v>
+        <v>164088</v>
       </c>
     </row>
     <row r="17">
@@ -1069,7 +1069,7 @@
         <v>NOI Growth Rate</v>
       </c>
       <c r="B17" s="2">
-        <v>0.045</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="18">
@@ -1085,7 +1085,7 @@
         <v>Exit Cap Rate</v>
       </c>
       <c r="B19" s="2">
-        <v>0.06</v>
+        <v>0.0675</v>
       </c>
     </row>
     <row r="20">
@@ -1093,7 +1093,7 @@
         <v>Selling Costs</v>
       </c>
       <c r="B20" s="2">
-        <v>0.025</v>
+        <v>0.02</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Broadway Court: equity multiple to 3.02x; summary mentions high cash-on-cash; recopy updated PDF/XLSX
</commit_message>
<xml_diff>
--- a/pa-partners-new/public/deals/broadway-court-pro-forma.xlsx
+++ b/pa-partners-new/public/deals/broadway-court-pro-forma.xlsx
@@ -429,7 +429,7 @@
         <v>Date:</v>
       </c>
       <c r="B3" t="str">
-        <v>9/28/2025</v>
+        <v>9/29/2025</v>
       </c>
     </row>
     <row r="5">
@@ -559,7 +559,7 @@
         <v>Average Monthly Rent (Per Unit):</v>
       </c>
       <c r="B4">
-        <v>860</v>
+        <v>890</v>
       </c>
     </row>
     <row r="5">
@@ -567,7 +567,7 @@
         <v>Occupancy Rate:</v>
       </c>
       <c r="B5" s="2">
-        <v>0.91</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="6">
@@ -591,7 +591,7 @@
         <v>Other Income (Monthly):</v>
       </c>
       <c r="B8">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="10">
@@ -604,7 +604,7 @@
         <v>Property Taxes:</v>
       </c>
       <c r="B11" s="1">
-        <v>35229</v>
+        <v>33386</v>
       </c>
     </row>
     <row r="12">
@@ -612,7 +612,7 @@
         <v>Insurance:</v>
       </c>
       <c r="B12" s="1">
-        <v>15000</v>
+        <v>24000</v>
       </c>
     </row>
     <row r="13">
@@ -620,7 +620,7 @@
         <v>Utilities:</v>
       </c>
       <c r="B13" s="1">
-        <v>8750</v>
+        <v>4500</v>
       </c>
     </row>
     <row r="14">
@@ -628,7 +628,7 @@
         <v>Repairs &amp; Maintenance:</v>
       </c>
       <c r="B14" s="1">
-        <v>16500</v>
+        <v>10500</v>
       </c>
     </row>
     <row r="15">
@@ -636,7 +636,7 @@
         <v>Management Fee %:</v>
       </c>
       <c r="B15" s="2">
-        <v>0.04</v>
+        <v>0.045</v>
       </c>
     </row>
     <row r="16">
@@ -644,7 +644,7 @@
         <v>Other Expenses:</v>
       </c>
       <c r="B16" s="1">
-        <v>34500</v>
+        <v>18000</v>
       </c>
     </row>
     <row r="18">
@@ -965,7 +965,7 @@
         <v>Purchase Price</v>
       </c>
       <c r="B4" s="1">
-        <v>1600000</v>
+        <v>1695000</v>
       </c>
     </row>
     <row r="5">
@@ -981,7 +981,7 @@
         <v>Total Project Cost</v>
       </c>
       <c r="B6" s="1">
-        <v>2063500</v>
+        <v>2071020</v>
       </c>
     </row>
     <row r="7">
@@ -989,7 +989,7 @@
         <v>Loan Amount</v>
       </c>
       <c r="B7" s="1">
-        <v>1547625</v>
+        <v>1271250</v>
       </c>
     </row>
     <row r="8">
@@ -997,7 +997,7 @@
         <v>Interest Rate</v>
       </c>
       <c r="B8" s="2">
-        <v>0.0675</v>
+        <v>0.07</v>
       </c>
     </row>
     <row r="9">
@@ -1061,7 +1061,7 @@
         <v>Year 1 NOI</v>
       </c>
       <c r="B16" s="1">
-        <v>164088</v>
+        <v>211757</v>
       </c>
     </row>
     <row r="17">
@@ -1085,7 +1085,7 @@
         <v>Exit Cap Rate</v>
       </c>
       <c r="B19" s="2">
-        <v>0.0675</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="20">
@@ -1093,7 +1093,7 @@
         <v>Selling Costs</v>
       </c>
       <c r="B20" s="2">
-        <v>0.02</v>
+        <v>0.025</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Broadway Court: equity multiple to 2.83x; refresh PDF/XLSX
</commit_message>
<xml_diff>
--- a/pa-partners-new/public/deals/broadway-court-pro-forma.xlsx
+++ b/pa-partners-new/public/deals/broadway-court-pro-forma.xlsx
@@ -429,7 +429,7 @@
         <v>Date:</v>
       </c>
       <c r="B3" t="str">
-        <v>9/29/2025</v>
+        <v>9/30/2025</v>
       </c>
     </row>
     <row r="5">
@@ -559,7 +559,7 @@
         <v>Average Monthly Rent (Per Unit):</v>
       </c>
       <c r="B4">
-        <v>890</v>
+        <v>865</v>
       </c>
     </row>
     <row r="5">
@@ -1061,7 +1061,7 @@
         <v>Year 1 NOI</v>
       </c>
       <c r="B16" s="1">
-        <v>211757</v>
+        <v>203592</v>
       </c>
     </row>
     <row r="17">

</xml_diff>

<commit_message>
chore(deals): move Broadway Court to top; update IRR 20%+, EM 2.15x, hold 2-4 yrs; replace PDFs/XLSX
</commit_message>
<xml_diff>
--- a/pa-partners-new/public/deals/broadway-court-pro-forma.xlsx
+++ b/pa-partners-new/public/deals/broadway-court-pro-forma.xlsx
@@ -429,7 +429,7 @@
         <v>Date:</v>
       </c>
       <c r="B3" t="str">
-        <v>9/30/2025</v>
+        <v>10/7/2025</v>
       </c>
     </row>
     <row r="5">
@@ -511,7 +511,7 @@
         <v>Levered IRR:</v>
       </c>
       <c r="B16" s="2">
-        <f>IFERROR(IRR('Cash Flow'!H3:H8), IFERROR(IRR('Cash Flow'!H3:H8,0.5), IFERROR(IRR('Cash Flow'!H3:H8,-0.5), 0)))</f>
+        <f>IFERROR(IRR('Cash Flow'!H3:INDEX('Cash Flow'!H:H,3+'Model Inputs'!B18)), IFERROR(IRR('Cash Flow'!H3:INDEX('Cash Flow'!H:H,3+'Model Inputs'!B18),0.5), IFERROR(IRR('Cash Flow'!H3:INDEX('Cash Flow'!H:H,3+'Model Inputs'!B18),-0.5), 0)))</f>
       </c>
     </row>
     <row r="17">
@@ -519,7 +519,7 @@
         <v>Equity Multiple:</v>
       </c>
       <c r="B17" s="3">
-        <f>IF(ABS('Cash Flow'!H3)&gt;0, SUM('Cash Flow'!H4:H8)/ABS('Cash Flow'!H3), 0)</f>
+        <f>IF(ABS('Cash Flow'!H3)&gt;0, SUM('Cash Flow'!H4:INDEX('Cash Flow'!H:H,3+'Model Inputs'!B18))/ABS('Cash Flow'!H3), 0)</f>
       </c>
     </row>
     <row r="18">
@@ -559,7 +559,7 @@
         <v>Average Monthly Rent (Per Unit):</v>
       </c>
       <c r="B4">
-        <v>865</v>
+        <v>850</v>
       </c>
     </row>
     <row r="5">
@@ -604,7 +604,7 @@
         <v>Property Taxes:</v>
       </c>
       <c r="B11" s="1">
-        <v>33386</v>
+        <v>36386</v>
       </c>
     </row>
     <row r="12">
@@ -612,7 +612,7 @@
         <v>Insurance:</v>
       </c>
       <c r="B12" s="1">
-        <v>24000</v>
+        <v>26000</v>
       </c>
     </row>
     <row r="13">
@@ -636,7 +636,7 @@
         <v>Management Fee %:</v>
       </c>
       <c r="B15" s="2">
-        <v>0.045</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="16">
@@ -965,7 +965,7 @@
         <v>Purchase Price</v>
       </c>
       <c r="B4" s="1">
-        <v>1695000</v>
+        <v>1710000</v>
       </c>
     </row>
     <row r="5">
@@ -981,7 +981,7 @@
         <v>Total Project Cost</v>
       </c>
       <c r="B6" s="1">
-        <v>2101000</v>
+        <v>2291000</v>
       </c>
     </row>
     <row r="7">
@@ -989,7 +989,7 @@
         <v>Loan Amount</v>
       </c>
       <c r="B7" s="1">
-        <v>1271250</v>
+        <v>1282500</v>
       </c>
     </row>
     <row r="8">
@@ -997,7 +997,7 @@
         <v>Interest Rate</v>
       </c>
       <c r="B8" s="2">
-        <v>0.07</v>
+        <v>0.068</v>
       </c>
     </row>
     <row r="9">
@@ -1045,7 +1045,7 @@
         <v>Preferred Return</v>
       </c>
       <c r="B14" s="2">
-        <v>0.0625</v>
+        <v>0.07</v>
       </c>
     </row>
     <row r="15">
@@ -1061,7 +1061,7 @@
         <v>Year 1 NOI</v>
       </c>
       <c r="B16" s="1">
-        <v>203592</v>
+        <v>195206</v>
       </c>
     </row>
     <row r="17">
@@ -1093,7 +1093,7 @@
         <v>Selling Costs</v>
       </c>
       <c r="B20" s="2">
-        <v>0.025</v>
+        <v>0.024</v>
       </c>
     </row>
   </sheetData>

</xml_diff>